<commit_message>
feat: Add FinSimCo Q2-Q4 runs, trade plan and final report
- Optimizer starts from current holdings with a trading cost, never sells
  positions below cost basis, and outputs a share-level trade plan
- Actual FinSimCo equity, leverage and margin rate set via env vars;
  holdings per quarter in data/holdings_<Q>.csv, news log in data/news.csv
- Master workbook with every quarter: outputs/simulaciones_finsimco.xlsx
- Spanish report on the decisions per quarter: informe_finsimco.pdf

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/06_optimizacion_sharpe/outputs/Q1/resultados_sharpe_Q1.xlsx
+++ b/06_optimizacion_sharpe/outputs/Q1/resultados_sharpe_Q1.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weights" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage weights" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset stats" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covariance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weights" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage summary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage weights" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset stats" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Covariance" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,62 +501,126 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dropped tickers</t>
+          <t>Strategy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>Equity</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.04</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Leverage</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>2</v>
+          <t>Equity source</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Initial capital</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Margin rate</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.04</v>
+        <v>199996346.1044</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Short rebate</t>
+          <t>Short</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.04</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Margin loan</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>99996346.10440001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Dropped tickers</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RF</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Leverage</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Margin rate</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Short rebate</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Borrow fee</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B19" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -570,72 +635,445 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Return</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Volatility</t>
+          <t>Weight (% equity)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Sharpe</t>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Prev shares</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Shares</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Trade shares</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Trade amount</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Max Sharpe</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.4401710751837257</v>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>0.09353197590901319</v>
+        <v>0.4909336565</v>
       </c>
       <c r="D2" t="n">
-        <v>4.278441370393024</v>
+        <v>266.35</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>184319</v>
+      </c>
+      <c r="G2" t="n">
+        <v>184319</v>
+      </c>
+      <c r="H2" t="n">
+        <v>49093365.65000001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>49093365.65000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Min variance</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.1804715439700959</v>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>0.06243442697699252</v>
+        <v>0.3772812251</v>
       </c>
       <c r="D3" t="n">
-        <v>2.249905232923185</v>
+        <v>165.23</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>228337</v>
+      </c>
+      <c r="G3" t="n">
+        <v>228337</v>
+      </c>
+      <c r="H3" t="n">
+        <v>37728122.51</v>
+      </c>
+      <c r="I3" t="n">
+        <v>37728122.51</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Equal weight</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.1834632789795839</v>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1165858311443348</v>
+        <v>0.2677024918</v>
       </c>
       <c r="D4" t="n">
-        <v>1.230537858429593</v>
+        <v>326.57</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>81974</v>
+      </c>
+      <c r="G4" t="n">
+        <v>81974</v>
+      </c>
+      <c r="H4" t="n">
+        <v>26770249.18</v>
+      </c>
+      <c r="I4" t="n">
+        <v>26770249.18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2222.SR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.226983612744</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7.0308</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3228418</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3228418</v>
+      </c>
+      <c r="H5" t="n">
+        <v>22698361.2744</v>
+      </c>
+      <c r="I5" t="n">
+        <v>22698361.2744</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>005930.KS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.178143812</v>
+      </c>
+      <c r="D6" t="n">
+        <v>215.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>82627</v>
+      </c>
+      <c r="G6" t="n">
+        <v>82627</v>
+      </c>
+      <c r="H6" t="n">
+        <v>17814381.2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>17814381.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.1309728997</v>
+      </c>
+      <c r="D7" t="n">
+        <v>428.03</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>30599</v>
+      </c>
+      <c r="G7" t="n">
+        <v>30599</v>
+      </c>
+      <c r="H7" t="n">
+        <v>13097289.97</v>
+      </c>
+      <c r="I7" t="n">
+        <v>13097289.97</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0871800093</v>
+      </c>
+      <c r="D8" t="n">
+        <v>330.39</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>26387</v>
+      </c>
+      <c r="G8" t="n">
+        <v>26387</v>
+      </c>
+      <c r="H8" t="n">
+        <v>8718000.93</v>
+      </c>
+      <c r="I8" t="n">
+        <v>8718000.93</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0633711788</v>
+      </c>
+      <c r="D9" t="n">
+        <v>388.28</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16321</v>
+      </c>
+      <c r="G9" t="n">
+        <v>16321</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6337117.88</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6337117.88</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0606735324</v>
+      </c>
+      <c r="D10" t="n">
+        <v>492.44</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>12321</v>
+      </c>
+      <c r="G10" t="n">
+        <v>12321</v>
+      </c>
+      <c r="H10" t="n">
+        <v>6067353.24</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6067353.24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0563557187</v>
+      </c>
+      <c r="D11" t="n">
+        <v>367.21</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15347</v>
+      </c>
+      <c r="G11" t="n">
+        <v>15347</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5635571.87</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5635571.87</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.05527406</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1123</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4922</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4922</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5527406</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5527406</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.005091264</v>
+      </c>
+      <c r="D13" t="n">
+        <v>353.56</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1440</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1440</v>
+      </c>
+      <c r="H13" t="n">
+        <v>509126.4</v>
+      </c>
+      <c r="I13" t="n">
+        <v>509126.4</v>
       </c>
     </row>
   </sheetData>
@@ -649,344 +1087,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Max Sharpe</t>
+          <t>Return</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Min variance</t>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Sharpe</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>Max Sharpe</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1338519061678334</v>
+        <v>0.4401710751837257</v>
       </c>
       <c r="C2" t="n">
-        <v>0.02264128006823838</v>
+        <v>0.09353197590901319</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4.278441370393024</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>Min variance</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.03033750095962639</v>
+        <v>0.1804715439700959</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02322763781589031</v>
+        <v>0.06243442697699252</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.249905232923185</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2222.SR</t>
+          <t>Equal weight</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1134918102687526</v>
+        <v>0.1834632789795839</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2428926730938863</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0.04359031453297787</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AMZN</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1.304772153889645e-13</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.01026359762959942</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>7.195306859757135e-06</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.03212422507427236</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.781646519522495e-13</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>BRK-B</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1.439751426642912e-13</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.2217803552969174</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1.722316994475595e-13</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.001321426590430233</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.0654871784879662</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.008225487919218441</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.02817858648108407</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.0541671293087318</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>UNH</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.0316859163302486</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.003438008035568616</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MC.PA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2.426062309416326e-13</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.02352914684174037</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>XOM</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.1886409242797062</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.09377882477853448</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TCEHY</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3.674932323236348e-13</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.004785153068757297</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>LLY</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.02764258685409551</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1.62575788470658e-18</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0.2454670943164866</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.079092394431132</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0.002546010172916183</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.01354261491169577</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WMT</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1.586557360038716e-13</v>
-      </c>
-      <c r="C20" t="n">
-        <v>0.03244663444802057</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>NVO</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1.927364567731199e-13</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0.008952337816256838</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1.3251213235885e-13</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1.398491834080968e-13</v>
-      </c>
-      <c r="C23" t="n">
-        <v>0.02215011367089988</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>PG</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>2.153177203847378e-13</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.05844358388846296</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>005930.KS</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>0.08907297583954313</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.03377660300833953</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3.21783469094529e-13</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0.009420772303407023</v>
+        <v>0.1165858311443348</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.230537858429593</v>
       </c>
     </row>
   </sheetData>
@@ -1000,156 +1166,344 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Return</t>
+          <t>Max Sharpe</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Volatility</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Sharpe</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Short</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Gross</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Borrowed</t>
+          <t>Min variance</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Max Sharpe (no leverage)</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4401710751837257</v>
+        <v>0.1338519061678334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.09353197590901319</v>
-      </c>
-      <c r="D2" t="n">
-        <v>4.278441370393024</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1.000000000000492</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1.000000000000492</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
+        <v>0.02264128006823838</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A. Levered max Sharpe (2x)</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.8403421503674514</v>
+        <v>0.03033750095962639</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1870639518180264</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4.278441370393024</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2.000000000000985</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2.000000000000985</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
+        <v>0.02322763781589031</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B. Long/short, no financing</t>
+          <t>2222.SR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.6716082495270052</v>
+        <v>0.1134918102687526</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1243045690433716</v>
-      </c>
-      <c r="D4" t="n">
-        <v>5.081134622707458</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1.499999999999999</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.4999999999999997</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1.999999999999999</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.4999999999999993</v>
+        <v>0.2428926730938863</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B. Long/short, rebate + 0.5% fee</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6716344940881852</v>
+        <v>0.04359031453297787</v>
       </c>
       <c r="C5" t="n">
-        <v>0.1248027238756107</v>
-      </c>
-      <c r="D5" t="n">
-        <v>5.061063368438393</v>
-      </c>
-      <c r="E5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.4999999999999997</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.5</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.304772153889645e-13</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.01026359762959942</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>7.195306859757135e-06</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.03212422507427236</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.781646519522495e-13</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BRK-B</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1.439751426642912e-13</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.2217803552969174</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1.722316994475595e-13</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.001321426590430233</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.0654871784879662</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.008225487919218441</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.02817858648108407</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0541671293087318</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.0316859163302486</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.003438008035568616</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MC.PA</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.426062309416326e-13</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.02352914684174037</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1886409242797062</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.09377882477853448</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TCEHY</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.674932323236348e-13</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.004785153068757297</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.02764258685409551</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.62575788470658e-18</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.2454670943164866</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.079092394431132</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.002546010172916183</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.01354261491169577</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1.586557360038716e-13</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.03244663444802057</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NVO</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1.927364567731199e-13</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.008952337816256838</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.3251213235885e-13</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.398491834080968e-13</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.02215011367089988</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2.153177203847378e-13</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.05844358388846296</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>005930.KS</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.08907297583954313</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.03377660300833953</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3.21783469094529e-13</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.009420772303407023</v>
       </c>
     </row>
   </sheetData>
@@ -1163,504 +1517,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Max Sharpe</t>
+          <t>Return</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>A. Levered</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>B. No financing</t>
+          <t>Sharpe</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>B. Rebate + fee</t>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Gross</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Borrowed</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>Max Sharpe (no leverage)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1338519061678334</v>
+        <v>0.4401710751837257</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2677038123356668</v>
+        <v>0.09353197590901319</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2089339465178185</v>
+        <v>4.278441370393024</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2099351924808575</v>
+        <v>1.000000000000492</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.000000000000492</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>A. Levered max Sharpe (2x)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.03033750095962639</v>
+        <v>0.8403421503674514</v>
       </c>
       <c r="C3" t="n">
-        <v>0.06067500191925278</v>
+        <v>0.1870639518180264</v>
       </c>
       <c r="D3" t="n">
-        <v>0.08110547691113543</v>
+        <v>4.278441370393024</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08102318493196821</v>
+        <v>2.000000000000985</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.000000000000985</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2222.SR</t>
+          <t>B. Long/short, no financing</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1134918102687526</v>
+        <v>0.6716082495270052</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2269836205375052</v>
+        <v>0.1243045690433716</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1577928812044403</v>
+        <v>5.081134622707458</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1566098487166108</v>
+        <v>1.499999999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.4999999999999997</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.999999999999999</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.4999999999999993</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>B. Long/short, rebate + 0.5% fee</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.04359031453297787</v>
+        <v>0.6716344940881852</v>
       </c>
       <c r="C5" t="n">
-        <v>0.08718062906595574</v>
+        <v>0.1248027238756107</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1230158992138084</v>
+        <v>5.061063368438393</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1236979014904925</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AMZN</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1.304772153889645e-13</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2.60954430777929e-13</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.002000816082144939</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.001922446730604932</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>7.195306859757135e-06</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1.439061371951427e-05</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.01537345879576515</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.01531330628702275</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.781646519522495e-13</v>
-      </c>
-      <c r="C8" t="n">
-        <v>3.563293039044991e-13</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-0.02886754141498527</v>
-      </c>
-      <c r="E8" t="n">
-        <v>-0.02874714296271538</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>BRK-B</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1.439751426642912e-13</v>
-      </c>
-      <c r="C9" t="n">
-        <v>2.879502853285823e-13</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>META</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1.722316994475595e-13</v>
-      </c>
-      <c r="C10" t="n">
-        <v>3.44463398895119e-13</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.002699422897231705</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.002412194014110728</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.0654871784879662</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.1309743569759324</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.1211992866241368</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.1216851297325109</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.02817858648108407</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.05635717296216815</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.05192140021864545</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.04946863700772065</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>UNH</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.0316859163302486</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.0633718326604972</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.0511058062827742</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.05122118195782734</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MC.PA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2.426062309416326e-13</v>
-      </c>
-      <c r="C14" t="n">
-        <v>4.852124618832653e-13</v>
-      </c>
-      <c r="D14" t="n">
-        <v>-0.03462307238213169</v>
-      </c>
-      <c r="E14" t="n">
-        <v>-0.03514208884804591</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>XOM</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.1886409242797062</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0.3772818485594123</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.2123099143648041</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.2129201183533502</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TCEHY</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>3.674932323236348e-13</v>
-      </c>
-      <c r="C16" t="n">
-        <v>7.349864646472695e-13</v>
-      </c>
-      <c r="D16" t="n">
-        <v>-0.1642861014716573</v>
-      </c>
-      <c r="E16" t="n">
-        <v>-0.1652357301041112</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>LLY</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.02764258685409551</v>
-      </c>
-      <c r="C17" t="n">
-        <v>0.05528517370819102</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.04325620643401468</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.04352999594612038</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>JNJ</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0.2454670943164866</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.4909341886329733</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.2985620824354433</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.2996399773557628</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>JPM</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>0.002546010172916183</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0.005092020345832366</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.03248121554252748</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.03183471193475432</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WMT</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1.586557360038716e-13</v>
-      </c>
-      <c r="C20" t="n">
-        <v>3.173114720077431e-13</v>
-      </c>
-      <c r="D20" t="n">
-        <v>-0.008726317180567367</v>
-      </c>
-      <c r="E20" t="n">
-        <v>-0.008592470844904771</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>NVO</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1.927364567731199e-13</v>
-      </c>
-      <c r="C21" t="n">
-        <v>3.854729135462399e-13</v>
-      </c>
-      <c r="D21" t="n">
-        <v>-0.01118198887617811</v>
-      </c>
-      <c r="E21" t="n">
-        <v>-0.01106862045663169</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>MA</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1.3251213235885e-13</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2.650242647177001e-13</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-0.03034458626517198</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-0.02793060733122216</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>AVGO</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1.398491834080968e-13</v>
-      </c>
-      <c r="C23" t="n">
-        <v>2.796983668161935e-13</v>
-      </c>
-      <c r="D23" t="n">
-        <v>-0.01900180501076272</v>
-      </c>
-      <c r="E23" t="n">
-        <v>-0.0188543220376675</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>PG</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>2.153177203847378e-13</v>
-      </c>
-      <c r="C24" t="n">
-        <v>4.306354407694755e-13</v>
-      </c>
-      <c r="D24" t="n">
-        <v>-0.1587596865548853</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-0.1598985022995955</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>005930.KS</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>0.08907297583954313</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.1781459516790863</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.09824218647530875</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.09878617306028591</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>ORCL</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>3.21783469094529e-13</v>
-      </c>
-      <c r="C26" t="n">
-        <v>6.43566938189058e-13</v>
-      </c>
-      <c r="D26" t="n">
-        <v>-0.0442089008436599</v>
-      </c>
-      <c r="E26" t="n">
-        <v>-0.04453051511510566</v>
+        <v>1.5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.4999999999999997</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -1674,424 +1680,504 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Annual return</t>
+          <t>Max Sharpe</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Annual volatility</t>
+          <t>A. Levered</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Sharpe</t>
+          <t>B. No financing</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>B. Rebate + fee</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>005930.KS</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.504931983427119</v>
+        <v>0.1338519061678334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7265846700426549</v>
+        <v>0.2677038123356668</v>
       </c>
       <c r="D2" t="n">
-        <v>2.016188950616201</v>
+        <v>0.2089339465178185</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2099351924808575</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JNJ</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3887136637893198</v>
+        <v>0.03033750095962639</v>
       </c>
       <c r="C3" t="n">
-        <v>0.185463256514055</v>
+        <v>0.06067500191925278</v>
       </c>
       <c r="D3" t="n">
-        <v>1.880230458278905</v>
+        <v>0.08110547691113543</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.08102318493196821</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>XOM</t>
+          <t>2222.SR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4070654588942863</v>
+        <v>0.1134918102687526</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2451521289880957</v>
+        <v>0.2269836205375052</v>
       </c>
       <c r="D4" t="n">
-        <v>1.497296639476097</v>
+        <v>0.1577928812044403</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.1566098487166108</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5805702577955969</v>
+        <v>0.04359031453297787</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3841440324942655</v>
+        <v>0.08718062906595574</v>
       </c>
       <c r="D5" t="n">
-        <v>1.407207224554937</v>
+        <v>0.1230158992138084</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.1236979014904925</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4450690821105578</v>
+        <v>1.304772153889645e-13</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3436333743127338</v>
+        <v>2.60954430777929e-13</v>
       </c>
       <c r="D6" t="n">
-        <v>1.178782715505138</v>
+        <v>0.002000816082144939</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.001922446730604932</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3216845162362933</v>
+        <v>7.195306859757135e-06</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2409458337274956</v>
+        <v>1.439061371951427e-05</v>
       </c>
       <c r="D7" t="n">
-        <v>1.16907817777365</v>
+        <v>0.01537345879576515</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.01531330628702275</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.361778005048402</v>
+        <v>1.781646519522495e-13</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2978871054635522</v>
+        <v>3.563293039044991e-13</v>
       </c>
       <c r="D8" t="n">
-        <v>1.080201187452113</v>
+        <v>-0.02886754141498527</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.02874714296271538</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>BRK-B</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.1960135750693193</v>
+        <v>1.439751426642912e-13</v>
       </c>
       <c r="C9" t="n">
-        <v>0.211007468538071</v>
+        <v>2.879502853285823e-13</v>
       </c>
       <c r="D9" t="n">
-        <v>0.7393746588698142</v>
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.3056200037564458</v>
+        <v>1.722316994475595e-13</v>
       </c>
       <c r="C10" t="n">
-        <v>0.3624637936214462</v>
+        <v>3.44463398895119e-13</v>
       </c>
       <c r="D10" t="n">
-        <v>0.7328180315682975</v>
+        <v>0.002699422897231705</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.002412194014110728</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.2378046175461348</v>
+        <v>0.0654871784879662</v>
       </c>
       <c r="C11" t="n">
-        <v>0.3406501404494569</v>
+        <v>0.1309743569759324</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5806679465481788</v>
+        <v>0.1211992866241368</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1216851297325109</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2222.SR</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1157448262775777</v>
+        <v>0.02817858648108407</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1498178056323528</v>
+        <v>0.05635717296216815</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5055796002209016</v>
+        <v>0.05192140021864545</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.04946863700772065</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TSLA</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1470191351042403</v>
+        <v>0.0316859163302486</v>
       </c>
       <c r="C13" t="n">
-        <v>0.4515640067552648</v>
+        <v>0.0633718326604972</v>
       </c>
       <c r="D13" t="n">
-        <v>0.2369966018178276</v>
+        <v>0.0511058062827742</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.05122118195782734</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>MC.PA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1137340846655421</v>
+        <v>2.426062309416326e-13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3295437761917922</v>
+        <v>4.852124618832653e-13</v>
       </c>
       <c r="D14" t="n">
-        <v>0.2237459481638925</v>
+        <v>-0.03462307238213169</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-0.03514208884804591</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>XOM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1399509707255866</v>
+        <v>0.1886409242797062</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4482048649000327</v>
+        <v>0.3772818485594123</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2230028688954092</v>
+        <v>0.2123099143648041</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.2129201183533502</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>TCEHY</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.08725027604933913</v>
+        <v>3.674932323236348e-13</v>
       </c>
       <c r="C16" t="n">
-        <v>0.2129030630661621</v>
+        <v>7.349864646472695e-13</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2219332844199407</v>
+        <v>-0.1642861014716573</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-0.1652357301041112</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WMT</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.06164355787939688</v>
+        <v>0.02764258685409551</v>
       </c>
       <c r="C17" t="n">
-        <v>0.2486279977231036</v>
+        <v>0.05528517370819102</v>
       </c>
       <c r="D17" t="n">
-        <v>0.08705197354121504</v>
+        <v>0.04325620643401468</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.04352999594612038</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>JNJ</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.03740675025754153</v>
+        <v>0.2454670943164866</v>
       </c>
       <c r="C18" t="n">
-        <v>0.3131166003607492</v>
+        <v>0.4909341886329733</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.008282057672671234</v>
+        <v>0.2985620824354433</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.2996399773557628</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BRK-B</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.03398380161148532</v>
+        <v>0.002546010172916183</v>
       </c>
       <c r="C19" t="n">
-        <v>0.1386431002985215</v>
+        <v>0.005092020345832366</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.04339342077291123</v>
+        <v>0.03248121554252748</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.03183471193475432</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.01081539740692161</v>
+        <v>1.586557360038716e-13</v>
       </c>
       <c r="C20" t="n">
-        <v>0.2157182181723539</v>
+        <v>3.173114720077431e-13</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.235563773136311</v>
+        <v>-0.008726317180567367</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-0.008592470844904771</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.0695055476833453</v>
+        <v>1.927364567731199e-13</v>
       </c>
       <c r="C21" t="n">
-        <v>0.3837299873922471</v>
+        <v>3.854729135462399e-13</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.2853713581977872</v>
+        <v>-0.01118198887617811</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-0.01106862045663169</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.09285326524209593</v>
+        <v>1.3251213235885e-13</v>
       </c>
       <c r="C22" t="n">
-        <v>0.445412113353934</v>
+        <v>2.650242647177001e-13</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.2982704359827948</v>
+        <v>-0.03034458626517198</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-0.02793060733122216</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.2072027559702382</v>
+        <v>1.398491834080968e-13</v>
       </c>
       <c r="C23" t="n">
-        <v>0.6550758610805492</v>
+        <v>2.796983668161935e-13</v>
       </c>
       <c r="D23" t="n">
-        <v>-0.3773650819043716</v>
+        <v>-0.01900180501076272</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-0.0188543220376675</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MC.PA</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.1314656397516503</v>
+        <v>2.153177203847378e-13</v>
       </c>
       <c r="C24" t="n">
-        <v>0.290730747137147</v>
+        <v>4.306354407694755e-13</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.5897747019883127</v>
+        <v>-0.1587596865548853</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-0.1598985022995955</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>005930.KS</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>-0.08045400675337511</v>
+        <v>0.08907297583954313</v>
       </c>
       <c r="C25" t="n">
-        <v>0.1884511465958087</v>
+        <v>0.1781459516790863</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.6391789539584265</v>
+        <v>0.09824218647530875</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.09878617306028591</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TCEHY</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.3071059789469596</v>
+        <v>3.21783469094529e-13</v>
       </c>
       <c r="C26" t="n">
-        <v>0.321873682759526</v>
+        <v>6.43566938189058e-13</v>
       </c>
       <c r="D26" t="n">
-        <v>-1.078391920616526</v>
+        <v>-0.0442089008436599</v>
+      </c>
+      <c r="E26" t="n">
+        <v>-0.04453051511510566</v>
       </c>
     </row>
   </sheetData>
@@ -2105,6 +2191,437 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Annual return</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Annual volatility</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Sharpe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>005930.KS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.504931983427119</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.7265846700426549</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.016188950616201</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>JNJ</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3887136637893198</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.185463256514055</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.880230458278905</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.4070654588942863</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.2451521289880957</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.497296639476097</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.5805702577955969</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3841440324942655</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.407207224554937</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.4450690821105578</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.3436333743127338</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.178782715505138</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.3216845162362933</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.2409458337274956</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.16907817777365</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.361778005048402</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.2978871054635522</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.080201187452113</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1960135750693193</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.211007468538071</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.7393746588698142</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3056200037564458</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.3624637936214462</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.7328180315682975</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2378046175461348</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3406501404494569</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5806679465481788</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2222.SR</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.1157448262775777</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.1498178056323528</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5055796002209016</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1470191351042403</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.4515640067552648</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.2369966018178276</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1137340846655421</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3295437761917922</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.2237459481638925</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1399509707255866</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.4482048649000327</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2230028688954092</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.08725027604933913</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2129030630661621</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.2219332844199407</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.06164355787939688</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.2486279977231036</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.08705197354121504</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.03740675025754153</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.3131166003607492</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-0.008282057672671234</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BRK-B</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.03398380161148532</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.1386431002985215</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.04339342077291123</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>-0.01081539740692161</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.2157182181723539</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.235563773136311</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>-0.0695055476833453</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.3837299873922471</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-0.2853713581977872</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>NVO</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>-0.09285326524209593</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.445412113353934</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-0.2982704359827948</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>-0.2072027559702382</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.6550758610805492</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-0.3773650819043716</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MC.PA</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>-0.1314656397516503</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.290730747137147</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-0.5897747019883127</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>-0.08045400675337511</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.1884511465958087</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.6391789539584265</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TCEHY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>-0.3071059789469596</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.321873682759526</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-1.078391920616526</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>